<commit_message>
Deployed 72299555 with MkDocs version: 1.6.0
</commit_message>
<xml_diff>
--- a/Manual/source/tab/parametersEN.xlsx
+++ b/Manual/source/tab/parametersEN.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="12"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="22"/>
   </bookViews>
   <sheets>
     <sheet name="TGZ-D-48-13_26" sheetId="1" state="visible" r:id="rId3"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1200" uniqueCount="292">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1200" uniqueCount="293">
   <si>
     <t xml:space="preserve">POWER SUPPLY</t>
   </si>
@@ -407,7 +407,7 @@
     <t xml:space="preserve">24 VDC ± 10 %, 600 mA*</t>
   </si>
   <si>
-    <t xml:space="preserve">0-320 VDC (pojistka 10 A)</t>
+    <t xml:space="preserve">0-320 VDC (fuse 10 A)</t>
   </si>
   <si>
     <t xml:space="preserve">2,6 kW</t>
@@ -417,6 +417,9 @@
   </si>
   <si>
     <t xml:space="preserve">2 x 10 A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LED signaling (axis 1 and 2 separately)</t>
   </si>
   <si>
     <t xml:space="preserve">1 x 3pin PHOENIX  PC 5/ 3-STCL1-7,62  </t>
@@ -1754,7 +1757,7 @@
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>31</v>
+        <v>124</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>32</v>
@@ -1773,7 +1776,7 @@
         <v>34</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1789,7 +1792,7 @@
         <v>38</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1852,7 +1855,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1969,7 +1972,7 @@
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>31</v>
+        <v>124</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>32</v>
@@ -1988,7 +1991,7 @@
         <v>34</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2004,7 +2007,7 @@
         <v>38</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2067,7 +2070,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2075,7 +2078,7 @@
         <v>6</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2083,7 +2086,7 @@
         <v>8</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2091,7 +2094,7 @@
         <v>12</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2104,10 +2107,10 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2219,7 +2222,7 @@
         <v>34</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2235,7 +2238,7 @@
         <v>38</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2260,7 +2263,7 @@
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B30" s="3"/>
     </row>
@@ -2269,7 +2272,7 @@
         <v>117</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -2316,7 +2319,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2324,7 +2327,7 @@
         <v>6</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2332,7 +2335,7 @@
         <v>8</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2353,10 +2356,10 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2468,7 +2471,7 @@
         <v>34</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2484,7 +2487,7 @@
         <v>38</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2509,7 +2512,7 @@
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B30" s="3"/>
     </row>
@@ -2518,7 +2521,7 @@
         <v>117</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -2565,7 +2568,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2573,7 +2576,7 @@
         <v>6</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2581,7 +2584,7 @@
         <v>8</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2589,7 +2592,7 @@
         <v>12</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2602,10 +2605,10 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2717,7 +2720,7 @@
         <v>34</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2733,7 +2736,7 @@
         <v>38</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2758,7 +2761,7 @@
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B30" s="3"/>
     </row>
@@ -2767,7 +2770,7 @@
         <v>117</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -2814,7 +2817,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2822,7 +2825,7 @@
         <v>6</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2830,7 +2833,7 @@
         <v>8</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2838,7 +2841,7 @@
         <v>12</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2846,15 +2849,15 @@
         <v>14</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2966,7 +2969,7 @@
         <v>34</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2982,7 +2985,7 @@
         <v>38</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3007,7 +3010,7 @@
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B30" s="3"/>
     </row>
@@ -3016,7 +3019,7 @@
         <v>117</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -3055,7 +3058,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3063,7 +3066,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3071,7 +3074,7 @@
         <v>6</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3079,7 +3082,7 @@
         <v>8</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3087,7 +3090,7 @@
         <v>10</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3103,7 +3106,7 @@
         <v>14</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3199,7 +3202,7 @@
         <v>34</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3207,7 +3210,7 @@
         <v>36</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3223,7 +3226,7 @@
         <v>52</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3231,7 +3234,7 @@
         <v>40</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3239,12 +3242,12 @@
         <v>42</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3252,7 +3255,7 @@
         <v>117</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
   </sheetData>
@@ -3289,91 +3292,91 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C9" s="3"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C11" s="3"/>
     </row>
@@ -3388,7 +3391,7 @@
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>1</v>
@@ -3396,18 +3399,18 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>185</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3423,12 +3426,12 @@
         <v>58</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>1</v>
@@ -3436,26 +3439,26 @@
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
   </sheetData>
@@ -3492,16 +3495,16 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>1</v>
@@ -3510,25 +3513,25 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>46</v>
@@ -3537,25 +3540,25 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>1</v>
@@ -3564,19 +3567,19 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C11" s="3"/>
     </row>
@@ -3591,7 +3594,7 @@
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>1</v>
@@ -3599,18 +3602,18 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>185</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3626,12 +3629,12 @@
         <v>58</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>1</v>
@@ -3642,12 +3645,12 @@
         <v>36</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>1</v>
@@ -3655,7 +3658,7 @@
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>1</v>
@@ -3663,10 +3666,10 @@
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
   </sheetData>
@@ -3929,21 +3932,21 @@
         <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>46</v>
@@ -3952,16 +3955,16 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>46</v>
@@ -3970,7 +3973,7 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>56</v>
@@ -3979,25 +3982,25 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C9" s="3"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>1</v>
@@ -4006,19 +4009,19 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C12" s="3"/>
     </row>
@@ -4033,7 +4036,7 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>1</v>
@@ -4041,18 +4044,18 @@
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>185</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4068,12 +4071,12 @@
         <v>58</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>1</v>
@@ -4084,47 +4087,47 @@
         <v>36</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
   </sheetData>
@@ -4161,28 +4164,28 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C4" s="3"/>
     </row>
@@ -4200,19 +4203,19 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C8" s="3"/>
     </row>
@@ -4227,28 +4230,28 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C12" s="3"/>
     </row>
@@ -4266,16 +4269,16 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C15" s="3"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>1</v>
@@ -4283,10 +4286,10 @@
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4294,15 +4297,15 @@
         <v>19</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
   </sheetData>
@@ -4339,28 +4342,28 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C4" s="3"/>
     </row>
@@ -4405,10 +4408,10 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C10" s="3"/>
     </row>
@@ -4426,10 +4429,10 @@
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C13" s="3"/>
     </row>
@@ -4438,7 +4441,7 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>1</v>
@@ -4447,7 +4450,7 @@
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>37</v>
@@ -4458,7 +4461,7 @@
         <v>19</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4519,28 +4522,28 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C4" s="3"/>
     </row>
@@ -4585,10 +4588,10 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C10" s="3"/>
     </row>
@@ -4606,10 +4609,10 @@
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C13" s="3"/>
     </row>
@@ -4618,7 +4621,7 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>1</v>
@@ -4630,7 +4633,7 @@
         <v>19</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4657,7 +4660,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.2"/>
@@ -4673,107 +4676,107 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>244</v>
-      </c>
-      <c r="K1" s="0" t="s">
         <v>245</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>246</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4781,16 +4784,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D4" s="1" t="n">
         <v>24</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F4" s="1" t="n">
         <v>2.05</v>
@@ -4816,16 +4819,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D5" s="1" t="n">
         <v>24</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F5" s="1" t="n">
         <v>2.05</v>
@@ -4851,16 +4854,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D6" s="1" t="n">
         <v>24</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F6" s="1" t="n">
         <v>2.05</v>
@@ -4886,16 +4889,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D7" s="1" t="n">
         <v>24</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F7" s="1" t="n">
         <v>2.05</v>
@@ -4921,16 +4924,16 @@
         <v>5</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D8" s="1" t="n">
         <v>24</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F8" s="1" t="n">
         <v>2.05</v>
@@ -4956,16 +4959,16 @@
         <v>6</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D9" s="1" t="n">
         <v>24</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F9" s="1" t="n">
         <v>2.05</v>
@@ -4991,16 +4994,16 @@
         <v>7</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D10" s="1" t="n">
         <v>24</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="F10" s="1" t="n">
         <v>1.25</v>
@@ -5026,16 +5029,16 @@
         <v>8</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D11" s="1" t="n">
         <v>24</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="F11" s="1" t="n">
         <v>1.25</v>
@@ -5055,18 +5058,6 @@
       <c r="K11" s="1" t="n">
         <v>50</v>
       </c>
-    </row>
-    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="0"/>
-      <c r="C19" s="0"/>
-      <c r="D19" s="0"/>
-      <c r="E19" s="0"/>
-      <c r="F19" s="0"/>
-      <c r="G19" s="0"/>
-      <c r="H19" s="0"/>
-      <c r="I19" s="0"/>
-      <c r="J19" s="0"/>
-      <c r="K19" s="0"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -5084,7 +5075,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.2"/>
@@ -5099,89 +5090,89 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>275</v>
-      </c>
-      <c r="I1" s="0" t="s">
         <v>276</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>277</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5201,7 +5192,7 @@
         <v>0.5</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>300</v>
@@ -5230,7 +5221,7 @@
         <v>0.5</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>300</v>
@@ -5259,7 +5250,7 @@
         <v>0.5</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>300</v>
@@ -5288,7 +5279,7 @@
         <v>0.5</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>300</v>
@@ -5317,7 +5308,7 @@
         <v>0.5</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>300</v>
@@ -5346,7 +5337,7 @@
         <v>0.5</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>300</v>
@@ -5357,16 +5348,6 @@
       <c r="I9" s="1" t="n">
         <v>10</v>
       </c>
-    </row>
-    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="0"/>
-      <c r="C19" s="0"/>
-      <c r="D19" s="0"/>
-      <c r="E19" s="0"/>
-      <c r="F19" s="0"/>
-      <c r="G19" s="0"/>
-      <c r="H19" s="0"/>
-      <c r="I19" s="0"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -5384,7 +5365,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.2"/>
@@ -5395,44 +5376,44 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>286</v>
-      </c>
-      <c r="D1" s="0" t="s">
         <v>287</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>288</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5440,7 +5421,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C4" s="1" t="n">
         <v>11</v>
@@ -5454,7 +5435,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C5" s="1" t="n">
         <v>11</v>
@@ -5462,11 +5443,6 @@
       <c r="D5" s="1" t="n">
         <v>22</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="0"/>
-      <c r="C13" s="0"/>
-      <c r="D13" s="0"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>